<commit_message>
Add dedicated helmet family surface
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GXnYR71FXD6d6TpXxgFVYe
</commit_message>
<xml_diff>
--- a/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
+++ b/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -4214,6 +4214,53 @@
         </is>
       </c>
       <c r="K74" t="inlineStr">
+        <is>
+          <t>חסר</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>מוצרי צריכה נוספים</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>קסדות</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>לבדוק</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
         <is>
           <t>חסר</t>
         </is>

</xml_diff>

<commit_message>
Move pesticides poisons permit to the other-permit category
Product-owner decision (2026-10-13, P2 decision backlog): the
pesticides row moves from "משרד הבריאות" to "אישור / רישיון אחר" in the
workbook. The result's category, referral and note now all point to the
same Ministry of Environmental Protection poisons permit.

The matrix was regenerated (one row changed; deterministic). The three
Wave-2 pesticide tests now expect the new category, a new consistency
test checks that the three agree, and registry rule 40 records the
move.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FUZRSyU1uvUFPN54LiegdN
</commit_message>
<xml_diff>
--- a/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
+++ b/data/FreighTime_Simple_Import_Requirements_Matrix.xlsx
@@ -2503,7 +2503,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>כן</t>
+          <t>לבדוק</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>לבדוק</t>
+          <t>כן</t>
         </is>
       </c>
       <c r="I39" s="4" t="n"/>

</xml_diff>